<commit_message>
Apply client cache-busting to EJS templates to prevent outdated JS execution
</commit_message>
<xml_diff>
--- a/datasets/complaints_dataset.xlsx
+++ b/datasets/complaints_dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3970,6 +3970,126 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>1</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>2</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>3</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>4</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>5</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>6</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Our street light has been flickering since last week and is now completely dark.</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: optimize complaint ML models, status transitions, duplicate cascades, and dashboard metrics
</commit_message>
<xml_diff>
--- a/datasets/complaints_dataset.xlsx
+++ b/datasets/complaints_dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D167"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Main pipeline burst near Ward 2, water flooding the road. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Drinking water pipeline leakage near school, urgent repair needed. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>since yesterday: Low water pressure in municipal tap for past three days. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Water supply contaminated with mud and smell. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -546,12 +546,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Request for new water connection in Block B. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -568,12 +568,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>this is serious: Water supply timing is irregular in Ward 1. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -590,17 +590,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Huge pothole in front of school is causing accidents. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Main road caved in near temple, road is blocked. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -634,17 +634,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>since yesterday: Road tarring peeling off near bus stop. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -656,17 +656,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Speed breaker paint is faded, causing accidents at night. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. Please check the issue.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -678,17 +678,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Need road sweeping on Block A road. Please fix it urgently.</t>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>this is serious: Request for repairing side walking path. (Ward 2)</t>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -722,17 +722,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>All street lights in Ward 4 are non-functional, dangerous at night. Located in Ward 3.</t>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. We have reported this before.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -744,17 +744,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dark street near community hall, high risk of theft. Please fix it please help.</t>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>since yesterday: Single street light flickering near temple. (Ward 5)</t>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Street light pole bent and leaning towards road. Located in Ward 1.</t>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -810,17 +810,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Request for extra street light pole near park. Please fix it urgently.</t>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -832,17 +832,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>this is serious: Request for timer switch installation on street lights. (Ward 3)</t>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) Please check the issue.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dead animal rotting in the drainage channel near market, foul smell. Located in Ward 4.</t>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Garbage accumulation near water source, high risk of disease outbreak. Please fix it please help.</t>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -898,17 +898,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>since yesterday: Garbage bin overflowing and not cleared for three days. (Ward 1)</t>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) We have reported this before.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Public toilet is blocked and overflowing. Located in Ward 2.</t>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -942,17 +942,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Plaza cleaning requested. Please fix it urgently.</t>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -964,17 +964,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>this is serious: Need more dustbins installed in market area. (Ward 4)</t>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -986,12 +986,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Blocked main sewer line causing sewage water to overflow onto streets. Located in Ward 5.</t>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Open manhole on main road, major hazard for kids. Please fix it please help.</t>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>since yesterday: Blocked storm water drain causing minor logging after rain. (Ward 2)</t>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1052,17 +1052,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Drainage cover cracked, needs replacement. Located in Ward 3.</t>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Drain cleaning requested before monsoon. Please fix it urgently.</t>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1096,17 +1096,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>this is serious: Request for laying closed drainage pipes in Block C. (Ward 5)</t>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1118,17 +1118,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Live electric wire hanging dangerously low near school gate. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1140,17 +1140,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Electric spark from transformer near houses. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1162,17 +1162,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>since yesterday: Flickering power line causing appliance issues. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Power outage in Block D for past 6 hours without explanation. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. Please check the issue.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1206,12 +1206,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Request for transformer fencing to prevent animal accidents. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>this is serious: Request for changing old electricity meter. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Stray dogs attacking school children near playground. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. We have reported this before.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1272,17 +1272,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Wild boar entry from forest area, destroying crops. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>since yesterday: Loud music played late at night in wedding hall. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Encroachment of public footpath by local vendors. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Request for library membership card process info. Please fix it urgently.</t>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1360,17 +1360,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>this is serious: Information needed on playground booking. (Ward 2)</t>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) Please check the issue.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1382,17 +1382,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Main pipeline burst near Ward 2, water flooding the road. Located in Ward 3.</t>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1404,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Drinking water pipeline leakage near school, urgent repair needed. Please fix it please help.</t>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1426,12 +1426,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>since yesterday: Low water pressure in municipal tap for past three days. (Ward 5)</t>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) We have reported this before.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Water supply contaminated with mud and smell. Located in Ward 1.</t>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Request for new water connection in Block B. Please fix it urgently.</t>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1492,17 +1492,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>this is serious: Water supply timing is irregular in Ward 1. (Ward 3)</t>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1514,17 +1514,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Huge pothole in front of school is causing accidents. Located in Ward 4.</t>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1536,17 +1536,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Main road caved in near temple, road is blocked. Please fix it please help.</t>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>since yesterday: Road tarring peeling off near bus stop. (Ward 1)</t>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1580,17 +1580,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Speed breaker paint is faded, causing accidents at night. Located in Ward 2.</t>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Need road sweeping on Block A road. Please fix it urgently.</t>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>this is serious: Request for repairing side walking path. (Ward 4)</t>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>All street lights in Ward 4 are non-functional, dangerous at night. Located in Ward 5.</t>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dark street near community hall, high risk of theft. Please fix it please help.</t>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1690,17 +1690,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>since yesterday: Single street light flickering near temple. (Ward 2)</t>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1712,17 +1712,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Street light pole bent and leaning towards road. Located in Ward 3.</t>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. Please check the issue.</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1734,17 +1734,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Request for extra street light pole near park. Please fix it urgently.</t>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>this is serious: Request for timer switch installation on street lights. (Ward 5)</t>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dead animal rotting in the drainage channel near market, foul smell. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. We have reported this before.</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Garbage accumulation near water source, high risk of disease outbreak. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1822,17 +1822,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>since yesterday: Garbage bin overflowing and not cleared for three days. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Public toilet is blocked and overflowing. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1866,12 +1866,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Plaza cleaning requested. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>this is serious: Need more dustbins installed in market area. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) Please check the issue.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Blocked main sewer line causing sewage water to overflow onto streets. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1932,17 +1932,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Open manhole on main road, major hazard for kids. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1954,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>since yesterday: Blocked storm water drain causing minor logging after rain. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) We have reported this before.</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1976,17 +1976,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Drainage cover cracked, needs replacement. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1998,17 +1998,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Drain cleaning requested before monsoon. Please fix it urgently.</t>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2020,17 +2020,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>this is serious: Request for laying closed drainage pipes in Block C. (Ward 2)</t>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2042,17 +2042,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Live electric wire hanging dangerously low near school gate. Located in Ward 3.</t>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2064,17 +2064,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Electric spark from transformer near houses. Please fix it please help.</t>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2086,12 +2086,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>since yesterday: Flickering power line causing appliance issues. (Ward 5)</t>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Power outage in Block D for past 6 hours without explanation. Located in Ward 1.</t>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Request for transformer fencing to prevent animal accidents. Please fix it urgently.</t>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2152,17 +2152,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>this is serious: Request for changing old electricity meter. (Ward 3)</t>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Stray dogs attacking school children near playground. Located in Ward 4.</t>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2196,17 +2196,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Wild boar entry from forest area, destroying crops. Please fix it please help.</t>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2218,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>since yesterday: Loud music played late at night in wedding hall. (Ward 1)</t>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2240,17 +2240,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Encroachment of public footpath by local vendors. Located in Ward 2.</t>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. Please check the issue.</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2262,17 +2262,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Request for library membership card process info. Please fix it urgently.</t>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2284,17 +2284,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>this is serious: Information needed on playground booking. (Ward 4)</t>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Main pipeline burst near Ward 2, water flooding the road. Located in Ward 5.</t>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. We have reported this before.</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Drinking water pipeline leakage near school, urgent repair needed. Please fix it please help.</t>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>since yesterday: Low water pressure in municipal tap for past three days. (Ward 2)</t>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2372,17 +2372,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Water supply contaminated with mud and smell. Located in Ward 3.</t>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2394,17 +2394,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Request for new water connection in Block B. Please fix it urgently.</t>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2416,17 +2416,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>this is serious: Water supply timing is irregular in Ward 1. (Ward 5)</t>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) Please check the issue.</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2438,17 +2438,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Huge pothole in front of school is causing accidents. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2460,17 +2460,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Main road caved in near temple, road is blocked. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2482,17 +2482,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>since yesterday: Road tarring peeling off near bus stop. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) We have reported this before.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2504,17 +2504,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Speed breaker paint is faded, causing accidents at night. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Need road sweeping on Block A road. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>this is serious: Request for repairing side walking path. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2570,17 +2570,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>All street lights in Ward 4 are non-functional, dangerous at night. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Dark street near community hall, high risk of theft. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2614,17 +2614,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>since yesterday: Single street light flickering near temple. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2636,17 +2636,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Street light pole bent and leaning towards road. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Request for extra street light pole near park. Please fix it urgently.</t>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2680,17 +2680,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>this is serious: Request for timer switch installation on street lights. (Ward 2)</t>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2702,17 +2702,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Dead animal rotting in the drainage channel near market, foul smell. Located in Ward 3.</t>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2724,17 +2724,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Garbage accumulation near water source, high risk of disease outbreak. Please fix it please help.</t>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2746,12 +2746,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>since yesterday: Garbage bin overflowing and not cleared for three days. (Ward 5)</t>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Public toilet is blocked and overflowing. Located in Ward 1.</t>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. Please check the issue.</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2790,17 +2790,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Plaza cleaning requested. Please fix it urgently.</t>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2812,17 +2812,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>this is serious: Need more dustbins installed in market area. (Ward 3)</t>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2834,17 +2834,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Blocked main sewer line causing sewage water to overflow onto streets. Located in Ward 4.</t>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. We have reported this before.</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Open manhole on main road, major hazard for kids. Please fix it please help.</t>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2878,17 +2878,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>since yesterday: Blocked storm water drain causing minor logging after rain. (Ward 1)</t>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2900,17 +2900,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Drainage cover cracked, needs replacement. Located in Ward 2.</t>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Drain cleaning requested before monsoon. Please fix it urgently.</t>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>this is serious: Request for laying closed drainage pipes in Block C. (Ward 4)</t>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) Please check the issue.</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Live electric wire hanging dangerously low near school gate. Located in Ward 5.</t>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2988,12 +2988,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Electric spark from transformer near houses. Please fix it please help.</t>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3010,17 +3010,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>since yesterday: Flickering power line causing appliance issues. (Ward 2)</t>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) We have reported this before.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Power outage in Block D for past 6 hours without explanation. Located in Ward 3.</t>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3054,17 +3054,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Request for transformer fencing to prevent animal accidents. Please fix it urgently.</t>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3076,17 +3076,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>this is serious: Request for changing old electricity meter. (Ward 5)</t>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3098,17 +3098,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Stray dogs attacking school children near playground. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3120,17 +3120,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Wild boar entry from forest area, destroying crops. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>since yesterday: Loud music played late at night in wedding hall. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3164,17 +3164,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Encroachment of public footpath by local vendors. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Request for library membership card process info. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>this is serious: Information needed on playground booking. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3230,17 +3230,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Main pipeline burst near Ward 2, water flooding the road. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3252,17 +3252,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Drinking water pipeline leakage near school, urgent repair needed. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3274,17 +3274,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>since yesterday: Low water pressure in municipal tap for past three days. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3296,17 +3296,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Water supply contaminated with mud and smell. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. Please check the issue.</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3318,17 +3318,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Request for new water connection in Block B. Please fix it urgently.</t>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Water Supply</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>this is serious: Water supply timing is irregular in Ward 1. (Ward 2)</t>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Huge pothole in front of school is causing accidents. Located in Ward 3.</t>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. We have reported this before.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Main road caved in near temple, road is blocked. Please fix it please help.</t>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3406,12 +3406,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>since yesterday: Road tarring peeling off near bus stop. (Ward 5)</t>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -3428,12 +3428,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Speed breaker paint is faded, causing accidents at night. Located in Ward 1.</t>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -3450,17 +3450,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Need road sweeping on Block A road. Please fix it urgently.</t>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Road Damage</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>this is serious: Request for repairing side walking path. (Ward 3)</t>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) Please check the issue.</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3494,17 +3494,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>All street lights in Ward 4 are non-functional, dangerous at night. Located in Ward 4.</t>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3516,17 +3516,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Dark street near community hall, high risk of theft. Please fix it please help.</t>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3538,17 +3538,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>since yesterday: Single street light flickering near temple. (Ward 1)</t>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) We have reported this before.</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3560,17 +3560,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Street light pole bent and leaning towards road. Located in Ward 2.</t>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3582,17 +3582,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Request for extra street light pole near park. Please fix it urgently.</t>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3604,17 +3604,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>this is serious: Request for timer switch installation on street lights. (Ward 4)</t>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Dead animal rotting in the drainage channel near market, foul smell. Located in Ward 5.</t>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -3648,12 +3648,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Garbage accumulation near water source, high risk of disease outbreak. Please fix it please help.</t>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. Please check the issue.</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -3670,17 +3670,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>since yesterday: Garbage bin overflowing and not cleared for three days. (Ward 2)</t>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) This has been a problem for days.</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Water Supply</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3692,17 +3692,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Public toilet is blocked and overflowing. Located in Ward 3.</t>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3714,17 +3714,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Plaza cleaning requested. Please fix it urgently.</t>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. We have reported this before.</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>this is serious: Need more dustbins installed in market area. (Ward 5)</t>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3758,17 +3758,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Blocked main sewer line causing sewage water to overflow onto streets. Located in Ward 1.</t>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3780,17 +3780,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Open manhole on main road, major hazard for kids. Please fix it please help.</t>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3802,17 +3802,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>since yesterday: Blocked storm water drain causing minor logging after rain. (Ward 3)</t>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) My name is citizen and I live here.</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3824,17 +3824,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Drainage cover cracked, needs replacement. Located in Ward 4.</t>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. Please check the issue.</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3846,12 +3846,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Drain cleaning requested before monsoon. Please fix it urgently.</t>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. This has been a problem for days.</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3868,12 +3868,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>this is serious: Request for laying closed drainage pipes in Block C. (Ward 1)</t>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) The panchayat officers must take action.</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3890,17 +3890,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Live electric wire hanging dangerously low near school gate. Located in Ward 2.</t>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. We have reported this before.</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3912,17 +3912,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Electric spark from transformer near houses. Please fix it please help.</t>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. Kindly resolve this at the earliest.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Road Damage</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3934,17 +3934,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>since yesterday: Flickering power line causing appliance issues. (Ward 4)</t>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) This is located near the landmark shop.</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Sanitation</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3956,135 +3956,895 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Power outage in Block D for past 6 hours without explanation. Located in Ward 5.</t>
+          <t>Request for library membership card procedure. Located in Ward 5. It is causing a lot of inconvenience to the residents.</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>C_SEED_161</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. My name is citizen and I live here.</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>C_SEED_162</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) Please check the issue.</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>C_SEED_163</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. This has been a problem for days.</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>C_SEED_164</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. The panchayat officers must take action.</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>C_SEED_165</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) We have reported this before.</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>C_SEED_166</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. Kindly resolve this at the earliest.</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>C_SEED_167</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. This is located near the landmark shop.</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
           <t>Electricity</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="n">
-        <v>1</v>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>C_SEED_168</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) It is causing a lot of inconvenience to the residents.</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>C_SEED_169</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. My name is citizen and I live here.</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>C_SEED_170</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. Please check the issue.</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>C_SEED_171</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>since yesterday: Main water pipeline burst near Ward 2, water flooding the road. (Ward 1) This has been a problem for days.</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>C_SEED_172</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Live electric wire hanging dangerously low near the school gate. Located in Ward 2. The panchayat officers must take action.</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>C_SEED_173</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Open manhole on the main road is a major safety hazard. Please fix it urgently. We have reported this before.</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>C_SEED_174</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>this is serious: Sewer drainage overflow onto public streets causing foul smell. (Ward 4) Kindly resolve this at the earliest.</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>C_SEED_175</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Electric sparks and transformer sparking near residential buildings. Located in Ward 5. This is located near the landmark shop.</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>C_SEED_176</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>A big tree has fallen down, blocking the main double road. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>C_SEED_177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>since yesterday: Drinking water pipe burst flooding the community ground. (Ward 2) My name is citizen and I live here.</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>C_SEED_178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Electric pole fallen onto the walking track causing danger. Located in Ward 3. Please check the issue.</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>C_SEED_179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Sewer manhole cover cracked and open near market. Please fix it urgently. This has been a problem for days.</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>C_SEED_180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>this is serious: Dead animal rotting in open drainage channel, toxic foul smell. (Ward 5) The panchayat officers must take action.</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>C_SEED_181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Request for installing a new dustbin in the market area. Located in Ward 1. We have reported this before.</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>C_SEED_182</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Please arrange for street sweeping on the main street. Please fix it please help. Kindly resolve this at the earliest.</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>C_SEED_183</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>since yesterday: Need general information on how to get a birth certificate. (Ward 3) This is located near the landmark shop.</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>C_SEED_184</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Minor cleaning issue near the local temple steps. Located in Ward 4. It is causing a lot of inconvenience to the residents.</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>C_SEED_185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Request for a new park bench or dustbin near Block B. Please fix it urgently. My name is citizen and I live here.</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>C_SEED_186</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>this is serious: Where can I find instructions on playground booking? (Ward 1) Please check the issue.</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>C_SEED_187</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>General query regarding the timing of Gram Sabha meeting. Located in Ward 2. This has been a problem for days.</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>C_SEED_188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Faded speed breaker paint needs minor touch up. Please fix it please help. The panchayat officers must take action.</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>C_SEED_189</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>since yesterday: Minor garbage cleaning requested near community hall. (Ward 4) We have reported this before.</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>C_SEED_190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Request for library membership card procedure. Located in Ward 5. Kindly resolve this at the earliest.</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>C_SEED_191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>The street light in our lane is not working and it is dark. Please fix it urgently. This is located near the landmark shop.</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
         <is>
           <t>Street Light</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="n">
-        <v>2</v>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>C_SEED_192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>this is serious: Low municipal water pressure in the taps for the past three days. (Ward 2) It is causing a lot of inconvenience to the residents.</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>C_SEED_193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Small potholes on the lane leading to the government school. Located in Ward 3. My name is citizen and I live here.</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>C_SEED_194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Road maintenance request for filling cracks on the walking path. Please fix it please help. Please check the issue.</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>C_SEED_195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>since yesterday: Single street light bulb flickering near the temple. (Ward 5) This has been a problem for days.</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
         <is>
           <t>Street Light</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="n">
-        <v>3</v>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Street Light</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="n">
-        <v>4</v>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Street Light</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="n">
-        <v>5</v>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Street Light</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="n">
-        <v>6</v>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>Our street light has been flickering since last week and is now completely dark.</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>Street Light</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>C_SEED_196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Municipal water supply is irregular in our block. Located in Ward 1. The panchayat officers must take action.</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Water Supply</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>C_SEED_197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Flickering electricity line causing appliance power issues. Please fix it urgently. We have reported this before.</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>C_SEED_198</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>this is serious: Tarring peeling off near the local bus stop. (Ward 3) Kindly resolve this at the earliest.</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Road Damage</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>C_SEED_199</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Garbage collection is delayed by a day. Located in Ward 4. This is located near the landmark shop.</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Sanitation</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>C_SEED_200</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Blocked storm water drain causing minor logging after rain. Please fix it please help. It is causing a lot of inconvenience to the residents.</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>